<commit_message>
Mise à jour site panneaux rocko
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rocko\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\rocko\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F020C9-7DB9-4E74-A412-9B99A91B337E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A5A3284-6F7D-4D77-AF51-E5223A41D895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -143,10 +143,10 @@
     <t>galerie/R130.jpg</t>
   </si>
   <si>
-    <t>1230x2800</t>
+    <t>galerie/R156.jpg</t>
   </si>
   <si>
-    <t>galerie/R156.jpg</t>
+    <t>1230x2800x0,4</t>
   </si>
 </sst>
 </file>
@@ -694,7 +694,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D2" s="6">
         <v>199.8</v>
@@ -714,7 +714,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D3" s="6">
         <v>199.8</v>
@@ -734,7 +734,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" s="6">
         <v>199.8</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D5" s="6">
         <v>199.8</v>
@@ -774,7 +774,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6">
         <v>199.8</v>
@@ -794,7 +794,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" s="6">
         <v>199.8</v>
@@ -808,13 +808,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" s="6">
         <v>199.8</v>
@@ -834,7 +834,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D9" s="6">
         <v>199.8</v>
@@ -854,7 +854,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="6">
         <v>199.8</v>
@@ -874,7 +874,7 @@
         <v>25</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" s="6">
         <v>199.8</v>

</xml_diff>